<commit_message>
Ajout de la struturation du projet
</commit_message>
<xml_diff>
--- a/exo_1_refait_05-03-2026_15-17.xlsx
+++ b/exo_1_refait_05-03-2026_15-17.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahmoud At-Tidianie\Desktop\GITHUB\Exo-de-donn-e-E-commerce-\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Données Brutes" sheetId="1" r:id="rId1"/>
     <sheet name="Données Néttoyées" sheetId="2" r:id="rId2"/>
     <sheet name="Données Par Catégories" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -438,11 +443,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -506,11 +511,19 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -552,7 +565,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -584,9 +597,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -618,6 +632,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -793,9 +808,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" customWidth="1"/>
@@ -812,7 +827,7 @@
     <col min="13" max="13" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -853,7 +868,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -894,7 +909,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -935,7 +950,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -976,7 +991,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1017,7 +1032,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1058,7 +1073,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1096,7 +1111,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1137,7 +1152,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1178,7 +1193,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1219,7 +1234,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1260,9 +1275,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" customWidth="1"/>
@@ -1274,13 +1289,13 @@
     <col min="8" max="8" width="11.7109375" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" customWidth="1"/>
     <col min="10" max="10" width="11.7109375" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.7109375" customWidth="1"/>
     <col min="13" max="13" width="12.7109375" customWidth="1"/>
     <col min="14" max="14" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1324,7 +1339,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1368,7 +1383,7 @@
         <v>899.99</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1412,7 +1427,7 @@
         <v>1999.98</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1456,7 +1471,7 @@
         <v>449.99</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1500,7 +1515,7 @@
         <v>599.97</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1544,7 +1559,7 @@
         <v>1299.99</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1588,7 +1603,7 @@
         <v>1199.98</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1632,7 +1647,7 @@
         <v>699.99</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1676,7 +1691,7 @@
         <v>899.99</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1720,7 +1735,7 @@
         <v>549.99</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1770,44 +1785,44 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>

</xml_diff>